<commit_message>
E14 parte 1: flecos de E13 (alternativo huérfano y Volver a AL 00, buscador del árbol físico y de la vista funcional) y demo corregida
- Baja de una fila que deja un único AL en su hueco: la confirmación ofrece volver a AL 00 (marcado),
  arrastrando el CS de las filas hijas; auditado. Observación OF-012 "Alternativo único" y botón
  "Volver a AL 00" en la ficha. El badge Alternativo solo con 2 AL o más.
- Árbol físico: buscador por SNS, nombre, NOC o P/N (el servidor da la ruta de CS de cada coincidencia),
  la abre, la resalta y navega "n de m"; Expandir / Contraer todo. Buscador también en la vista funcional.
- demo/CONFUNFIS_DEMO_TRAMONTANA.xlsx: unidad de medida L -> LI en productos funcionales.
- verify-confunfis: buscar segmentos y silentblock; borrar la copia vuelve a AL 00.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0144hBQAzKGxu1EtSHETQ5V4
</commit_message>
<xml_diff>
--- a/demo/CONFUNFIS_DEMO_TRAMONTANA.xlsx
+++ b/demo/CONFUNFIS_DEMO_TRAMONTANA.xlsx
@@ -4592,7 +4592,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>LI</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>LI</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>LI</t>
         </is>
       </c>
     </row>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>LI</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4792,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>LI</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>LI</t>
         </is>
       </c>
     </row>
@@ -4942,7 +4942,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>LI</t>
         </is>
       </c>
     </row>

</xml_diff>